<commit_message>
fix(sample): add msre to data template
</commit_message>
<xml_diff>
--- a/bioinformatics-analysis/resources/data-meta-en.xlsx
+++ b/bioinformatics-analysis/resources/data-meta-en.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P31"/>
+  <dimension ref="A1:Q31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="10.33203125" bestFit="1" customWidth="1" style="7" min="3" max="3"/>
@@ -609,6 +609,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Data Name Of R2</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr" s="1">
+        <is>
+          <t>MSRE</t>
         </is>
       </c>
     </row>

</xml_diff>